<commit_message>
chore: sync Nova upm-release-2026.10.10-01
</commit_message>
<xml_diff>
--- a/Assets/Samples/AppsflyerDemo/Excels/UIs/UIs.xlsx
+++ b/Assets/Samples/AppsflyerDemo/Excels/UIs/UIs.xlsx
@@ -1339,7 +1339,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:G48"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultColWidth="14" defaultRowHeight="14" outlineLevelCol="6"/>
   <cols>
     <col min="1" max="1" width="11.2115384615385" style="4" customWidth="1"/>
@@ -1424,17 +1424,25 @@
       </c>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:7">
-      <c r="B5" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>20</v>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>DemoAppsflyerView</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Appsflyer 演示 Demo 视图</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>DemoAppsflyerView</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Demo</t>
+        </is>
       </c>
       <c r="F5" s="5" t="b">
         <v>0</v>
@@ -1443,714 +1451,6 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" ht="22" customHeight="1" spans="1:7">
-      <c r="B6" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F6" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G6" s="5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" ht="22" customHeight="1" spans="1:7">
-      <c r="B7" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F7" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G7" s="5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" ht="22" customHeight="1" spans="1:7">
-      <c r="B8" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F8" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G8" s="5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1" spans="1:7">
-      <c r="B9" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F9" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G9" s="5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" ht="22" customHeight="1" spans="1:7">
-      <c r="B10" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F10" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G10" s="5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" ht="22" customHeight="1" spans="1:7">
-      <c r="B11" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F11" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G11" s="5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" ht="22" customHeight="1" spans="1:7">
-      <c r="B12" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F12" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G12" s="5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" ht="22" customHeight="1" spans="1:7">
-      <c r="B13" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F13" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G13" s="5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" ht="22" customHeight="1" spans="1:7">
-      <c r="B14" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F14" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G14" s="5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" ht="22" customHeight="1" spans="1:7">
-      <c r="B15" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F15" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G15" s="5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" ht="22" customHeight="1" spans="1:7">
-      <c r="B16" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="E16" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F16" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G16" s="5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" ht="22" customHeight="1" spans="2:7">
-      <c r="B17" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F17" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G17" s="5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" ht="22" customHeight="1" spans="2:7">
-      <c r="B18" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="C18" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="E18" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F18" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G18" s="5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" ht="22" customHeight="1" spans="2:7">
-      <c r="B19" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="E19" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F19" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G19" s="5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" ht="22" customHeight="1" spans="2:7">
-      <c r="B20" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="C20" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="E20" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F20" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G20" s="5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" ht="22" customHeight="1" spans="2:7">
-      <c r="B21" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="C21" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="D21" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="E21" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F21" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G21" s="5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" ht="22" customHeight="1" spans="2:7">
-      <c r="B22" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="C22" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="E22" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F22" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G22" s="5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" ht="22" customHeight="1" spans="2:7">
-      <c r="B23" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="C23" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="D23" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="E23" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F23" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G23" s="5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" ht="22" customHeight="1" spans="2:7">
-      <c r="B24" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="C24" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="D24" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="E24" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F24" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G24" s="5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" ht="22" customHeight="1" spans="2:7">
-      <c r="B25" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="C25" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="D25" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="E25" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F25" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G25" s="5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" ht="22" customHeight="1" spans="2:7">
-      <c r="B26" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="C26" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="D26" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="E26" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F26" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G26" s="5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" ht="22" customHeight="1" spans="2:7">
-      <c r="B27" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="C27" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="D27" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="E27" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F27" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G27" s="5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" ht="22" customHeight="1" spans="2:7">
-      <c r="B28" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="C28" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="D28" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="E28" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F28" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G28" s="5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" ht="22" customHeight="1" spans="2:7">
-      <c r="B29" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="C29" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="D29" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="E29" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F29" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G29" s="5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" ht="22" customHeight="1" spans="2:7">
-      <c r="B30" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="C30" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="D30" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="E30" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F30" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G30" s="5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" ht="22" customHeight="1" spans="2:7">
-      <c r="B31" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="C31" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="D31" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="E31" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F31" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G31" s="5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" ht="22" customHeight="1" spans="2:7">
-      <c r="B32" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="C32" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="D32" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="E32" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F32" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G32" s="5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" ht="22" customHeight="1" spans="2:7">
-      <c r="B33" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="C33" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="D33" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="E33" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F33" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G33" s="5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" ht="22" customHeight="1" spans="2:7">
-      <c r="B34" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="C34" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="D34" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="E34" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F34" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G34" s="5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" ht="22" customHeight="1" spans="2:7">
-      <c r="B35" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="C35" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="D35" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="E35" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F35" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G35" s="5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" ht="22" customHeight="1" spans="2:7">
-      <c r="B36" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="C36" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="D36" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="E36" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F36" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G36" s="5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" ht="22" customHeight="1" spans="2:7">
-      <c r="B37" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="C37" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="D37" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="E37" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F37" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G37" s="5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" ht="22" customHeight="1" spans="2:7">
-      <c r="B38" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="C38" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="D38" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="E38" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F38" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G38" s="5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" ht="22" customHeight="1" spans="2:7">
-      <c r="B39" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="C39" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="D39" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="E39" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="F39" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G39" s="5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40" ht="22" customHeight="1" spans="2:7">
-      <c r="B40" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="C40" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="D40" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="E40" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="F40" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G40" s="5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41" ht="22" customHeight="1"/>
-    <row r="42" ht="22" customHeight="1"/>
-    <row r="43" ht="22" customHeight="1"/>
-    <row r="44" ht="22" customHeight="1"/>
-    <row r="45" ht="22" customHeight="1"/>
-    <row r="46" ht="22" customHeight="1"/>
-    <row r="47" ht="22" customHeight="1"/>
-    <row r="48" ht="22" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>